<commit_message>
docs: adiciona imagens e finaliza documentação do projeto
</commit_message>
<xml_diff>
--- a/Carteira_Inteligente.xlsx
+++ b/Carteira_Inteligente.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TI - Faculdade_Cursos_e_Treinamentos\Santander Excel com IA e Claude\Carteira Inteligente\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TI - Faculdade_Cursos_e_Treinamentos\Santander Excel com IA e Claude\Carteira Inteligente\carteira-inteligente-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B150627-3E51-4176-9B7F-D1951554AB10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34A5FE3-4B1C-4B94-BF79-7339FAE088E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5775" yWindow="1680" windowWidth="21600" windowHeight="13125" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
+    <workbookView xWindow="3555" yWindow="1710" windowWidth="21600" windowHeight="13125" activeTab="2" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
   </bookViews>
   <sheets>
     <sheet name="SIMULADOR" sheetId="2" r:id="rId1"/>
@@ -19,15 +19,15 @@
     <sheet name="DADOS" sheetId="5" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="investimento_mensal">SIMULADOR!$H$12</definedName>
-    <definedName name="patrimonio_acumulado">SIMULADOR!$H$22</definedName>
-    <definedName name="percentual_investir">SIMULADOR!$H$10</definedName>
-    <definedName name="periodo_investimento">SIMULADOR!$H$16</definedName>
-    <definedName name="renda_estimada">SIMULADOR!$H$26</definedName>
-    <definedName name="renda_mensal">SIMULADOR!$H$8</definedName>
-    <definedName name="rendimento_obtido">SIMULADOR!$H$24</definedName>
-    <definedName name="taxa_mensal">SIMULADOR!$H$14</definedName>
-    <definedName name="total_investido">SIMULADOR!$H$20</definedName>
+    <definedName name="investimento_mensal">SIMULADOR!$H$17</definedName>
+    <definedName name="patrimonio_acumulado">SIMULADOR!$H$27</definedName>
+    <definedName name="percentual_investir">SIMULADOR!$H$15</definedName>
+    <definedName name="periodo_investimento">SIMULADOR!$H$21</definedName>
+    <definedName name="renda_estimada">SIMULADOR!$H$31</definedName>
+    <definedName name="renda_mensal">SIMULADOR!$H$13</definedName>
+    <definedName name="rendimento_obtido">SIMULADOR!$H$29</definedName>
+    <definedName name="taxa_mensal">SIMULADOR!$H$19</definedName>
+    <definedName name="total_investido">SIMULADOR!$H$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -603,6 +603,31 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -615,9 +640,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -626,26 +648,28 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -670,30 +694,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -799,7 +799,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>CENÁRIOS!$C$6</c:f>
+              <c:f>CENÁRIOS!$C$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -834,7 +834,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>CENÁRIOS!$B$7:$B$11</c:f>
+              <c:f>CENÁRIOS!$B$12:$B$16</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -857,7 +857,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CENÁRIOS!$C$7:$C$11</c:f>
+              <c:f>CENÁRIOS!$C$12:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>"R$"#,##0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -891,7 +891,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>CENÁRIOS!$D$6</c:f>
+              <c:f>CENÁRIOS!$D$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -926,7 +926,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>CENÁRIOS!$B$7:$B$11</c:f>
+              <c:f>CENÁRIOS!$B$12:$B$16</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -949,7 +949,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CENÁRIOS!$D$7:$D$11</c:f>
+              <c:f>CENÁRIOS!$D$12:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>"R$"#,##0.00_);[Red]\("R$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1249,7 +1249,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>PERFIL!$E$8</c:f>
+              <c:f>PERFIL!$E$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1633,7 +1633,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>PERFIL!$B$9:$B$12</c:f>
+              <c:f>PERFIL!$B$14:$B$17</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1653,7 +1653,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>PERFIL!$E$9:$E$12</c:f>
+              <c:f>PERFIL!$E$14:$E$17</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
@@ -2874,17 +2874,72 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F67F1B52-27B4-AE0D-5118-1F5B037850EB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619124" y="171450"/>
+          <a:ext cx="4991101" cy="1666874"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>600074</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1057274</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>123826</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2910,23 +2965,73 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28574</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2ECA6EEA-7C7D-469B-A272-22C688970118}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="190500"/>
+          <a:ext cx="4991101" cy="1666874"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>571499</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1809749</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:colOff>2009775</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2949,6 +3054,56 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9526</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28574</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DAFA29B-9DF5-44C3-82EC-C2263D82A471}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="190500"/>
+          <a:ext cx="4991101" cy="1666874"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3271,7 +3426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1874DCC7-29C5-4FCA-A3A8-49FB95C01093}">
-  <dimension ref="A2:J26"/>
+  <dimension ref="A7:J31"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="9.140625" customWidth="1"/>
@@ -3284,198 +3439,198 @@
     <col min="11" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-    </row>
-    <row r="3" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="24" t="s">
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-    </row>
-    <row r="6" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="26" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+    </row>
+    <row r="11" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-    </row>
-    <row r="7" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+    </row>
+    <row r="12" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="27">
+      <c r="H13" s="33">
         <v>5000</v>
       </c>
-      <c r="I8" s="28"/>
-    </row>
-    <row r="9" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
+      <c r="I13" s="34"/>
+    </row>
+    <row r="14" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="6"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="29">
+      <c r="H15" s="25">
         <v>0.1</v>
       </c>
-      <c r="I10" s="30"/>
-    </row>
-    <row r="11" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="6"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="6" t="s">
+      <c r="I15" s="26"/>
+    </row>
+    <row r="16" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="31">
+      <c r="H17" s="24">
         <f>renda_mensal*percentual_investir</f>
         <v>500</v>
       </c>
-      <c r="I12" s="31"/>
-    </row>
-    <row r="13" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="6"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="6" t="s">
+      <c r="I17" s="24"/>
+    </row>
+    <row r="18" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="6"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="29">
+      <c r="H19" s="25">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="I14" s="30"/>
-    </row>
-    <row r="15" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="6" t="s">
+      <c r="I19" s="26"/>
+    </row>
+    <row r="20" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="32">
+      <c r="H21" s="27">
         <v>2</v>
       </c>
-      <c r="I16" s="33"/>
-    </row>
-    <row r="18" spans="2:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="26" t="s">
+      <c r="I21" s="28"/>
+    </row>
+    <row r="23" spans="2:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-    </row>
-    <row r="19" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="6" t="s">
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+    </row>
+    <row r="24" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H20" s="31">
+      <c r="H25" s="24">
         <f>investimento_mensal*12*periodo_investimento</f>
         <v>12000</v>
       </c>
-      <c r="I20" s="31"/>
-    </row>
-    <row r="21" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="6"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="6" t="s">
+      <c r="I25" s="24"/>
+    </row>
+    <row r="26" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="6"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H22" s="34">
+      <c r="H27" s="22">
         <f>FV(taxa_mensal,periodo_investimento*12,-investimento_mensal,0,0)</f>
         <v>13171.577555559783</v>
       </c>
-      <c r="I22" s="34"/>
-    </row>
-    <row r="23" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="6"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="6" t="s">
+      <c r="I27" s="22"/>
+    </row>
+    <row r="28" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="6"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H24" s="34">
+      <c r="H29" s="22">
         <f>patrimonio_acumulado-total_investido</f>
         <v>1171.5775555597829</v>
       </c>
-      <c r="I24" s="34"/>
-    </row>
-    <row r="25" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="6"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="6" t="s">
+      <c r="I29" s="22"/>
+    </row>
+    <row r="30" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="6"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H26" s="34">
+      <c r="H31" s="22">
         <f>patrimonio_acumulado*taxa_mensal</f>
         <v>105.37262044447827</v>
       </c>
-      <c r="I26" s="34"/>
+      <c r="I31" s="22"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H27:I27"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2D69112-01B2-4FBD-B688-7D45ACB01A88}">
-  <dimension ref="A2:G34"/>
+  <dimension ref="A7:G16"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -3488,191 +3643,172 @@
     <col min="8" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-    </row>
-    <row r="3" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="24" t="s">
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+    </row>
+    <row r="8" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="10" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E11" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F11" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B12" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="7">
-        <f>investimento_mensal*12*A7</f>
+      <c r="C12" s="7">
+        <f>investimento_mensal*12*A12</f>
         <v>12000</v>
       </c>
-      <c r="D7" s="8">
-        <f>FV(taxa_mensal,A7*12,-investimento_mensal,0,0)</f>
+      <c r="D12" s="8">
+        <f>FV(taxa_mensal,A12*12,-investimento_mensal,0,0)</f>
         <v>13171.577555559783</v>
       </c>
-      <c r="E7" s="8">
-        <f>D7-C7</f>
+      <c r="E12" s="8">
+        <f>D12-C12</f>
         <v>1171.5775555597829</v>
       </c>
-      <c r="F7" s="13">
-        <f>D7*taxa_mensal</f>
+      <c r="F12" s="13">
+        <f>D12*taxa_mensal</f>
         <v>105.37262044447827</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="15">
         <v>5</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="7">
-        <f>investimento_mensal*12*A8</f>
+      <c r="C13" s="7">
+        <f>investimento_mensal*12*A13</f>
         <v>30000</v>
       </c>
-      <c r="D8" s="8">
-        <f>FV(taxa_mensal,A8*12,-investimento_mensal,0,0)</f>
+      <c r="D13" s="8">
+        <f>FV(taxa_mensal,A13*12,-investimento_mensal,0,0)</f>
         <v>38311.933415940111</v>
       </c>
-      <c r="E8" s="9">
-        <f>D8-C8</f>
+      <c r="E13" s="9">
+        <f>D13-C13</f>
         <v>8311.9334159401114</v>
       </c>
-      <c r="F8" s="13">
-        <f>D8*taxa_mensal</f>
+      <c r="F13" s="13">
+        <f>D13*taxa_mensal</f>
         <v>306.49546732752088</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="15">
         <v>10</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B14" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="7">
-        <f>investimento_mensal*12*A9</f>
+      <c r="C14" s="7">
+        <f>investimento_mensal*12*A14</f>
         <v>60000</v>
       </c>
-      <c r="D9" s="8">
-        <f>FV(taxa_mensal,A9*12,-investimento_mensal,0,0)</f>
+      <c r="D14" s="8">
+        <f>FV(taxa_mensal,A14*12,-investimento_mensal,0,0)</f>
         <v>100108.73470495906</v>
       </c>
-      <c r="E9" s="9">
-        <f t="shared" ref="E9:E11" si="0">D9-C9</f>
+      <c r="E14" s="9">
+        <f t="shared" ref="E14" si="0">D14-C14</f>
         <v>40108.734704959061</v>
       </c>
-      <c r="F9" s="13">
-        <f>D9*taxa_mensal</f>
+      <c r="F14" s="13">
+        <f>D14*taxa_mensal</f>
         <v>800.8698776396725</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="15">
         <v>20</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B15" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="7">
-        <f>investimento_mensal*12*A10</f>
+      <c r="C15" s="7">
+        <f>investimento_mensal*12*A15</f>
         <v>120000</v>
       </c>
-      <c r="D10" s="8">
-        <f>FV(taxa_mensal,A10*12,-investimento_mensal,0,0)</f>
+      <c r="D15" s="8">
+        <f>FV(taxa_mensal,A15*12,-investimento_mensal,0,0)</f>
         <v>360565.60963756416</v>
       </c>
-      <c r="E10" s="9">
-        <f>D10-C10</f>
+      <c r="E15" s="9">
+        <f>D15-C15</f>
         <v>240565.60963756416</v>
       </c>
-      <c r="F10" s="13">
-        <f>D10*taxa_mensal</f>
+      <c r="F15" s="13">
+        <f>D15*taxa_mensal</f>
         <v>2884.5248771005135</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
         <v>30</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B16" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="19">
-        <f>investimento_mensal*12*A11</f>
+      <c r="C16" s="19">
+        <f>investimento_mensal*12*A16</f>
         <v>180000</v>
       </c>
-      <c r="D11" s="20">
-        <f>FV(taxa_mensal,A11*12,-investimento_mensal,0,0)</f>
+      <c r="D16" s="20">
+        <f>FV(taxa_mensal,A16*12,-investimento_mensal,0,0)</f>
         <v>1038206.6156855426</v>
       </c>
-      <c r="E11" s="14">
-        <f>D11-C11</f>
+      <c r="E16" s="14">
+        <f>D16-C16</f>
         <v>858206.61568554258</v>
       </c>
-      <c r="F11" s="21">
-        <f>D11*taxa_mensal</f>
+      <c r="F16" s="21">
+        <f>D16*taxa_mensal</f>
         <v>8305.6529254843408</v>
       </c>
     </row>
-    <row r="17" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="19" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="20" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="23" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="24" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="25" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="26" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="27" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="30" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="31" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="32" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="33" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="2">
-    <mergeCell ref="B2:F3"/>
-    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F8"/>
+    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -3681,7 +3817,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAA5817-F1A8-4485-9F20-7AE9EFCE1C82}">
-  <dimension ref="A2:G14"/>
+  <dimension ref="A7:G19"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -3689,145 +3825,144 @@
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="4.42578125" customWidth="1"/>
     <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="27.140625" customWidth="1"/>
+    <col min="6" max="6" width="30.5703125" customWidth="1"/>
     <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-    </row>
-    <row r="3" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-    </row>
-    <row r="4" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="24" t="s">
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+    </row>
+    <row r="8" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+    </row>
+    <row r="9" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-    </row>
-    <row r="5" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:6" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="40" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+    </row>
+    <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="2:6" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="38" t="s">
+      <c r="C11" s="48"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="39"/>
-    </row>
-    <row r="7" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="35" t="s">
+      <c r="F11" s="47"/>
+    </row>
+    <row r="12" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36" t="s">
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="37"/>
-    </row>
-    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="46" t="s">
+      <c r="F13" s="45"/>
+    </row>
+    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="42">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B9,DADOS!$B$3:$B$6,0),MATCH($E$6,DADOS!$C$2:$E$2,0))</f>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="39">
+        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B14,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F9" s="43"/>
-    </row>
-    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="46" t="s">
+      <c r="F14" s="40"/>
+    </row>
+    <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="42">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B10,DADOS!$B$3:$B$6,0),MATCH($E$6,DADOS!$C$2:$E$2,0))</f>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="39">
+        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B15,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.25</v>
       </c>
-      <c r="F10" s="43"/>
-    </row>
-    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46" t="s">
+      <c r="F15" s="40"/>
+    </row>
+    <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="42">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B11,DADOS!$B$3:$B$6,0),MATCH($E$6,DADOS!$C$2:$E$2,0))</f>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="39">
+        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B16,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.35</v>
       </c>
-      <c r="F11" s="43"/>
-    </row>
-    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="46" t="s">
+      <c r="F16" s="40"/>
+    </row>
+    <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="42">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B12,DADOS!$B$3:$B$6,0),MATCH($E$6,DADOS!$C$2:$E$2,0))</f>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="39">
+        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B17,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F12" s="43"/>
-    </row>
-    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="48" t="s">
+      <c r="F17" s="40"/>
+    </row>
+    <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="44">
-        <f>SUM(E9:E12)</f>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="41">
+        <f>SUM(E14:E17)</f>
         <v>1</v>
       </c>
-      <c r="F13" s="45"/>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C14" s="3"/>
+      <c r="F18" s="42"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C19" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B7:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B2:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6" xr:uid="{E0102A38-0475-4B80-AF4E-1F2610E84CEB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{E0102A38-0475-4B80-AF4E-1F2610E84CEB}">
       <formula1>"Conservador,Moderado,Agressivo"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: atualiza planilha Carteira Inteligente
</commit_message>
<xml_diff>
--- a/Carteira_Inteligente.xlsx
+++ b/Carteira_Inteligente.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TI - Faculdade_Cursos_e_Treinamentos\Santander Excel com IA e Claude\Carteira Inteligente\carteira-inteligente-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34A5FE3-4B1C-4B94-BF79-7339FAE088E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A19883-F99B-4A31-91B4-7A5884221312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3555" yWindow="1710" windowWidth="21600" windowHeight="13125" activeTab="2" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
   </bookViews>
   <sheets>
     <sheet name="SIMULADOR" sheetId="2" r:id="rId1"/>
@@ -603,31 +603,6 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -640,6 +615,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -648,29 +626,27 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -694,6 +670,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -862,19 +862,19 @@
                 <c:formatCode>"R$"#,##0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
+                  <c:v>2400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>12000</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>30000</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>60000</c:v>
-                </c:pt>
                 <c:pt idx="3">
-                  <c:v>120000</c:v>
+                  <c:v>24000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>180000</c:v>
+                  <c:v>36000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -954,19 +954,19 @@
                 <c:formatCode>"R$"#,##0.00_);[Red]\("R$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>13171.577555559783</c:v>
+                  <c:v>2634.3155111119563</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>38311.933415940111</c:v>
+                  <c:v>7662.3866831880223</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100108.73470495906</c:v>
+                  <c:v>20021.746940991812</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360565.60963756416</c:v>
+                  <c:v>72113.121927512839</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1038206.6156855426</c:v>
+                  <c:v>207641.32313710853</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3440,61 +3440,61 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="33">
-        <v>5000</v>
-      </c>
-      <c r="I13" s="34"/>
+      <c r="H13" s="27">
+        <v>1000</v>
+      </c>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
@@ -3503,10 +3503,10 @@
       <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="29">
         <v>0.1</v>
       </c>
-      <c r="I15" s="26"/>
+      <c r="I15" s="30"/>
     </row>
     <row r="16" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -3515,11 +3515,11 @@
       <c r="B17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="32">
         <f>renda_mensal*percentual_investir</f>
-        <v>500</v>
-      </c>
-      <c r="I17" s="24"/>
+        <v>100</v>
+      </c>
+      <c r="I17" s="32"/>
     </row>
     <row r="18" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6"/>
@@ -3528,10 +3528,10 @@
       <c r="B19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="25">
+      <c r="H19" s="29">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="I19" s="26"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
@@ -3540,33 +3540,33 @@
       <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="27">
+      <c r="H21" s="33">
         <v>2</v>
       </c>
-      <c r="I21" s="28"/>
+      <c r="I21" s="34"/>
     </row>
     <row r="23" spans="2:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
     </row>
     <row r="24" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="32">
         <f>investimento_mensal*12*periodo_investimento</f>
-        <v>12000</v>
-      </c>
-      <c r="I25" s="24"/>
+        <v>2400</v>
+      </c>
+      <c r="I25" s="32"/>
     </row>
     <row r="26" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6"/>
@@ -3575,11 +3575,11 @@
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="31">
         <f>FV(taxa_mensal,periodo_investimento*12,-investimento_mensal,0,0)</f>
-        <v>13171.577555559783</v>
-      </c>
-      <c r="I27" s="22"/>
+        <v>2634.3155111119563</v>
+      </c>
+      <c r="I27" s="31"/>
     </row>
     <row r="28" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6"/>
@@ -3588,11 +3588,11 @@
       <c r="B29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H29" s="22">
+      <c r="H29" s="31">
         <f>patrimonio_acumulado-total_investido</f>
-        <v>1171.5775555597829</v>
-      </c>
-      <c r="I29" s="22"/>
+        <v>234.31551111195631</v>
+      </c>
+      <c r="I29" s="31"/>
     </row>
     <row r="30" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6"/>
@@ -3601,19 +3601,14 @@
       <c r="B31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="31">
         <f>patrimonio_acumulado*taxa_mensal</f>
-        <v>105.37262044447827</v>
-      </c>
-      <c r="I31" s="22"/>
+        <v>21.07452408889565</v>
+      </c>
+      <c r="I31" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B7:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H15:I15"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="B23:I23"/>
@@ -3622,6 +3617,11 @@
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H15:I15"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -3644,29 +3644,29 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
@@ -3694,19 +3694,19 @@
       </c>
       <c r="C12" s="7">
         <f>investimento_mensal*12*A12</f>
-        <v>12000</v>
+        <v>2400</v>
       </c>
       <c r="D12" s="8">
         <f>FV(taxa_mensal,A12*12,-investimento_mensal,0,0)</f>
-        <v>13171.577555559783</v>
+        <v>2634.3155111119563</v>
       </c>
       <c r="E12" s="8">
         <f>D12-C12</f>
-        <v>1171.5775555597829</v>
+        <v>234.31551111195631</v>
       </c>
       <c r="F12" s="13">
         <f>D12*taxa_mensal</f>
-        <v>105.37262044447827</v>
+        <v>21.07452408889565</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -3718,19 +3718,19 @@
       </c>
       <c r="C13" s="7">
         <f>investimento_mensal*12*A13</f>
-        <v>30000</v>
+        <v>6000</v>
       </c>
       <c r="D13" s="8">
         <f>FV(taxa_mensal,A13*12,-investimento_mensal,0,0)</f>
-        <v>38311.933415940111</v>
+        <v>7662.3866831880223</v>
       </c>
       <c r="E13" s="9">
         <f>D13-C13</f>
-        <v>8311.9334159401114</v>
+        <v>1662.3866831880223</v>
       </c>
       <c r="F13" s="13">
         <f>D13*taxa_mensal</f>
-        <v>306.49546732752088</v>
+        <v>61.299093465504178</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -3742,19 +3742,19 @@
       </c>
       <c r="C14" s="7">
         <f>investimento_mensal*12*A14</f>
-        <v>60000</v>
+        <v>12000</v>
       </c>
       <c r="D14" s="8">
         <f>FV(taxa_mensal,A14*12,-investimento_mensal,0,0)</f>
-        <v>100108.73470495906</v>
+        <v>20021.746940991812</v>
       </c>
       <c r="E14" s="9">
         <f t="shared" ref="E14" si="0">D14-C14</f>
-        <v>40108.734704959061</v>
+        <v>8021.7469409918122</v>
       </c>
       <c r="F14" s="13">
         <f>D14*taxa_mensal</f>
-        <v>800.8698776396725</v>
+        <v>160.17397552793449</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -3766,19 +3766,19 @@
       </c>
       <c r="C15" s="7">
         <f>investimento_mensal*12*A15</f>
-        <v>120000</v>
+        <v>24000</v>
       </c>
       <c r="D15" s="8">
         <f>FV(taxa_mensal,A15*12,-investimento_mensal,0,0)</f>
-        <v>360565.60963756416</v>
+        <v>72113.121927512839</v>
       </c>
       <c r="E15" s="9">
         <f>D15-C15</f>
-        <v>240565.60963756416</v>
+        <v>48113.121927512839</v>
       </c>
       <c r="F15" s="13">
         <f>D15*taxa_mensal</f>
-        <v>2884.5248771005135</v>
+        <v>576.90497542010269</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -3790,19 +3790,19 @@
       </c>
       <c r="C16" s="19">
         <f>investimento_mensal*12*A16</f>
-        <v>180000</v>
+        <v>36000</v>
       </c>
       <c r="D16" s="20">
         <f>FV(taxa_mensal,A16*12,-investimento_mensal,0,0)</f>
-        <v>1038206.6156855426</v>
+        <v>207641.32313710853</v>
       </c>
       <c r="E16" s="14">
         <f>D16-C16</f>
-        <v>858206.61568554258</v>
+        <v>171641.32313710853</v>
       </c>
       <c r="F16" s="21">
         <f>D16*taxa_mensal</f>
-        <v>8305.6529254843408</v>
+        <v>1661.1305850968683</v>
       </c>
     </row>
   </sheetData>
@@ -3831,135 +3831,135 @@
   </cols>
   <sheetData>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:6" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="46" t="s">
+      <c r="C11" s="40"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="47"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44" t="s">
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="45"/>
+      <c r="F13" s="37"/>
     </row>
     <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="39">
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="42">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B14,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F14" s="40"/>
+      <c r="F14" s="43"/>
     </row>
     <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="39">
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="42">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B15,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.25</v>
       </c>
-      <c r="F15" s="40"/>
+      <c r="F15" s="43"/>
     </row>
     <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="39">
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="42">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B16,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.35</v>
       </c>
-      <c r="F16" s="40"/>
+      <c r="F16" s="43"/>
     </row>
     <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="39">
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="42">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B17,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F17" s="40"/>
+      <c r="F17" s="43"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="41">
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="44">
         <f>SUM(E14:E17)</f>
         <v>1</v>
       </c>
-      <c r="F18" s="42"/>
+      <c r="F18" s="45"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="B7:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{E0102A38-0475-4B80-AF4E-1F2610E84CEB}">

</xml_diff>

<commit_message>
docs: atualiza exemplo de renda mensal na planilha
</commit_message>
<xml_diff>
--- a/Carteira_Inteligente.xlsx
+++ b/Carteira_Inteligente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TI - Faculdade_Cursos_e_Treinamentos\Santander Excel com IA e Claude\Carteira Inteligente\carteira-inteligente-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A19883-F99B-4A31-91B4-7A5884221312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522D50AE-C3CE-4BAF-B009-78B33AB3D862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
   </bookViews>
@@ -603,6 +603,31 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -615,9 +640,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -626,27 +648,29 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -670,30 +694,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -862,19 +862,19 @@
                 <c:formatCode>"R$"#,##0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2400</c:v>
+                  <c:v>12000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6000</c:v>
+                  <c:v>30000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12000</c:v>
+                  <c:v>60000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>24000</c:v>
+                  <c:v>120000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>36000</c:v>
+                  <c:v>180000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -954,19 +954,19 @@
                 <c:formatCode>"R$"#,##0.00_);[Red]\("R$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2634.3155111119563</c:v>
+                  <c:v>13171.577555559783</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7662.3866831880223</c:v>
+                  <c:v>38311.933415940111</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20021.746940991812</c:v>
+                  <c:v>100108.73470495906</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>72113.121927512839</c:v>
+                  <c:v>360565.60963756416</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>207641.32313710853</c:v>
+                  <c:v>1038206.6156855426</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3440,61 +3440,61 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
     </row>
     <row r="11" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="27">
-        <v>1000</v>
-      </c>
-      <c r="I13" s="28"/>
+      <c r="H13" s="33">
+        <v>5000</v>
+      </c>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
@@ -3503,10 +3503,10 @@
       <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H15" s="29">
+      <c r="H15" s="25">
         <v>0.1</v>
       </c>
-      <c r="I15" s="30"/>
+      <c r="I15" s="26"/>
     </row>
     <row r="16" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -3515,11 +3515,11 @@
       <c r="B17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="32">
+      <c r="H17" s="24">
         <f>renda_mensal*percentual_investir</f>
-        <v>100</v>
-      </c>
-      <c r="I17" s="32"/>
+        <v>500</v>
+      </c>
+      <c r="I17" s="24"/>
     </row>
     <row r="18" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6"/>
@@ -3528,10 +3528,10 @@
       <c r="B19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="29">
+      <c r="H19" s="25">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="I19" s="30"/>
+      <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
@@ -3540,33 +3540,33 @@
       <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="33">
+      <c r="H21" s="27">
         <v>2</v>
       </c>
-      <c r="I21" s="34"/>
+      <c r="I21" s="28"/>
     </row>
     <row r="23" spans="2:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
     </row>
     <row r="24" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H25" s="32">
+      <c r="H25" s="24">
         <f>investimento_mensal*12*periodo_investimento</f>
-        <v>2400</v>
-      </c>
-      <c r="I25" s="32"/>
+        <v>12000</v>
+      </c>
+      <c r="I25" s="24"/>
     </row>
     <row r="26" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6"/>
@@ -3575,11 +3575,11 @@
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="31">
+      <c r="H27" s="22">
         <f>FV(taxa_mensal,periodo_investimento*12,-investimento_mensal,0,0)</f>
-        <v>2634.3155111119563</v>
-      </c>
-      <c r="I27" s="31"/>
+        <v>13171.577555559783</v>
+      </c>
+      <c r="I27" s="22"/>
     </row>
     <row r="28" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6"/>
@@ -3588,11 +3588,11 @@
       <c r="B29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H29" s="31">
+      <c r="H29" s="22">
         <f>patrimonio_acumulado-total_investido</f>
-        <v>234.31551111195631</v>
-      </c>
-      <c r="I29" s="31"/>
+        <v>1171.5775555597829</v>
+      </c>
+      <c r="I29" s="22"/>
     </row>
     <row r="30" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6"/>
@@ -3601,14 +3601,19 @@
       <c r="B31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H31" s="31">
+      <c r="H31" s="22">
         <f>patrimonio_acumulado*taxa_mensal</f>
-        <v>21.07452408889565</v>
-      </c>
-      <c r="I31" s="31"/>
+        <v>105.37262044447827</v>
+      </c>
+      <c r="I31" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H15:I15"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="B23:I23"/>
@@ -3617,11 +3622,6 @@
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="H27:I27"/>
-    <mergeCell ref="B7:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H15:I15"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -3644,29 +3644,29 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
     </row>
     <row r="8" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
@@ -3694,19 +3694,19 @@
       </c>
       <c r="C12" s="7">
         <f>investimento_mensal*12*A12</f>
-        <v>2400</v>
+        <v>12000</v>
       </c>
       <c r="D12" s="8">
         <f>FV(taxa_mensal,A12*12,-investimento_mensal,0,0)</f>
-        <v>2634.3155111119563</v>
+        <v>13171.577555559783</v>
       </c>
       <c r="E12" s="8">
         <f>D12-C12</f>
-        <v>234.31551111195631</v>
+        <v>1171.5775555597829</v>
       </c>
       <c r="F12" s="13">
         <f>D12*taxa_mensal</f>
-        <v>21.07452408889565</v>
+        <v>105.37262044447827</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -3718,19 +3718,19 @@
       </c>
       <c r="C13" s="7">
         <f>investimento_mensal*12*A13</f>
-        <v>6000</v>
+        <v>30000</v>
       </c>
       <c r="D13" s="8">
         <f>FV(taxa_mensal,A13*12,-investimento_mensal,0,0)</f>
-        <v>7662.3866831880223</v>
+        <v>38311.933415940111</v>
       </c>
       <c r="E13" s="9">
         <f>D13-C13</f>
-        <v>1662.3866831880223</v>
+        <v>8311.9334159401114</v>
       </c>
       <c r="F13" s="13">
         <f>D13*taxa_mensal</f>
-        <v>61.299093465504178</v>
+        <v>306.49546732752088</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -3742,19 +3742,19 @@
       </c>
       <c r="C14" s="7">
         <f>investimento_mensal*12*A14</f>
-        <v>12000</v>
+        <v>60000</v>
       </c>
       <c r="D14" s="8">
         <f>FV(taxa_mensal,A14*12,-investimento_mensal,0,0)</f>
-        <v>20021.746940991812</v>
+        <v>100108.73470495906</v>
       </c>
       <c r="E14" s="9">
         <f t="shared" ref="E14" si="0">D14-C14</f>
-        <v>8021.7469409918122</v>
+        <v>40108.734704959061</v>
       </c>
       <c r="F14" s="13">
         <f>D14*taxa_mensal</f>
-        <v>160.17397552793449</v>
+        <v>800.8698776396725</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -3766,19 +3766,19 @@
       </c>
       <c r="C15" s="7">
         <f>investimento_mensal*12*A15</f>
-        <v>24000</v>
+        <v>120000</v>
       </c>
       <c r="D15" s="8">
         <f>FV(taxa_mensal,A15*12,-investimento_mensal,0,0)</f>
-        <v>72113.121927512839</v>
+        <v>360565.60963756416</v>
       </c>
       <c r="E15" s="9">
         <f>D15-C15</f>
-        <v>48113.121927512839</v>
+        <v>240565.60963756416</v>
       </c>
       <c r="F15" s="13">
         <f>D15*taxa_mensal</f>
-        <v>576.90497542010269</v>
+        <v>2884.5248771005135</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -3790,19 +3790,19 @@
       </c>
       <c r="C16" s="19">
         <f>investimento_mensal*12*A16</f>
-        <v>36000</v>
+        <v>180000</v>
       </c>
       <c r="D16" s="20">
         <f>FV(taxa_mensal,A16*12,-investimento_mensal,0,0)</f>
-        <v>207641.32313710853</v>
+        <v>1038206.6156855426</v>
       </c>
       <c r="E16" s="14">
         <f>D16-C16</f>
-        <v>171641.32313710853</v>
+        <v>858206.61568554258</v>
       </c>
       <c r="F16" s="21">
         <f>D16*taxa_mensal</f>
-        <v>1661.1305850968683</v>
+        <v>8305.6529254843408</v>
       </c>
     </row>
   </sheetData>
@@ -3831,135 +3831,135 @@
   </cols>
   <sheetData>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
     </row>
     <row r="8" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="9" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
     </row>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:6" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="38" t="s">
+      <c r="C11" s="48"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="39"/>
+      <c r="F11" s="47"/>
     </row>
     <row r="12" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36" t="s">
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="37"/>
+      <c r="F13" s="45"/>
     </row>
     <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="42">
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="39">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B14,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F14" s="43"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="42">
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="39">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B15,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.25</v>
       </c>
-      <c r="F15" s="43"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="42">
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="39">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B16,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.35</v>
       </c>
-      <c r="F16" s="43"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="42">
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="39">
         <f>INDEX(DADOS!$C$3:$E$6,MATCH(B17,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
         <v>0.2</v>
       </c>
-      <c r="F17" s="43"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="49"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="44">
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="41">
         <f>SUM(E14:E17)</f>
         <v>1</v>
       </c>
-      <c r="F18" s="45"/>
+      <c r="F18" s="42"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
     <mergeCell ref="B7:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{E0102A38-0475-4B80-AF4E-1F2610E84CEB}">

</xml_diff>

<commit_message>
docs: atualiza formulas e versao final da planilha
</commit_message>
<xml_diff>
--- a/Carteira_Inteligente.xlsx
+++ b/Carteira_Inteligente.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TI - Faculdade_Cursos_e_Treinamentos\Santander Excel com IA e Claude\Carteira Inteligente\carteira-inteligente-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522D50AE-C3CE-4BAF-B009-78B33AB3D862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7FCCCF-1E17-48FB-BD55-5BDD17ECF598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
+    <workbookView xWindow="4860" yWindow="225" windowWidth="21600" windowHeight="14130" xr2:uid="{A57CD098-14EC-4185-B074-C651832BE373}"/>
   </bookViews>
   <sheets>
     <sheet name="SIMULADOR" sheetId="2" r:id="rId1"/>
@@ -603,31 +603,6 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -640,6 +615,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -648,29 +626,27 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -694,6 +670,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1658,16 +1658,16 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.2</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.35</c:v>
+                  <c:v>0.05</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3440,61 +3440,61 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="33">
+      <c r="H13" s="27">
         <v>5000</v>
       </c>
-      <c r="I13" s="34"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
@@ -3503,10 +3503,10 @@
       <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="29">
         <v>0.1</v>
       </c>
-      <c r="I15" s="26"/>
+      <c r="I15" s="30"/>
     </row>
     <row r="16" spans="1:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -3515,11 +3515,11 @@
       <c r="B17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="32">
         <f>renda_mensal*percentual_investir</f>
         <v>500</v>
       </c>
-      <c r="I17" s="24"/>
+      <c r="I17" s="32"/>
     </row>
     <row r="18" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6"/>
@@ -3528,10 +3528,10 @@
       <c r="B19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="25">
+      <c r="H19" s="29">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="I19" s="26"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
@@ -3540,33 +3540,33 @@
       <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="27">
+      <c r="H21" s="33">
         <v>2</v>
       </c>
-      <c r="I21" s="28"/>
+      <c r="I21" s="34"/>
     </row>
     <row r="23" spans="2:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
     </row>
     <row r="24" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="32">
         <f>investimento_mensal*12*periodo_investimento</f>
         <v>12000</v>
       </c>
-      <c r="I25" s="24"/>
+      <c r="I25" s="32"/>
     </row>
     <row r="26" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6"/>
@@ -3575,11 +3575,11 @@
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="31">
         <f>FV(taxa_mensal,periodo_investimento*12,-investimento_mensal,0,0)</f>
         <v>13171.577555559783</v>
       </c>
-      <c r="I27" s="22"/>
+      <c r="I27" s="31"/>
     </row>
     <row r="28" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6"/>
@@ -3588,11 +3588,11 @@
       <c r="B29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H29" s="22">
+      <c r="H29" s="31">
         <f>patrimonio_acumulado-total_investido</f>
         <v>1171.5775555597829</v>
       </c>
-      <c r="I29" s="22"/>
+      <c r="I29" s="31"/>
     </row>
     <row r="30" spans="2:9" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6"/>
@@ -3601,19 +3601,15 @@
       <c r="B31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="31">
         <f>patrimonio_acumulado*taxa_mensal</f>
         <v>105.37262044447827</v>
       </c>
-      <c r="I31" s="22"/>
+      <c r="I31" s="31"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="B7:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H15:I15"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="B23:I23"/>
@@ -3622,6 +3618,11 @@
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H15:I15"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -3644,29 +3645,29 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
@@ -3806,6 +3807,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="2">
     <mergeCell ref="B7:F8"/>
     <mergeCell ref="B9:F9"/>
@@ -3831,135 +3833,136 @@
   </cols>
   <sheetData>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:6" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="47"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="2:6" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44" t="s">
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="45"/>
+      <c r="F13" s="37"/>
     </row>
     <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="39">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B14,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
-        <v>0.2</v>
-      </c>
-      <c r="F14" s="40"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="42">
+        <f>VLOOKUP(B14,DADOS!$B$3:$E$6,MATCH($E$11,DADOS!$B$2:$E$2,0),FALSE)</f>
+        <v>0.7</v>
+      </c>
+      <c r="F14" s="43"/>
     </row>
     <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="39">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B15,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
-        <v>0.25</v>
-      </c>
-      <c r="F15" s="40"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="42">
+        <f>VLOOKUP(B15,DADOS!$B$3:$E$6,MATCH($E$11,DADOS!$B$2:$E$2,0),FALSE)</f>
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="43"/>
     </row>
     <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="39">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B16,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
-        <v>0.35</v>
-      </c>
-      <c r="F16" s="40"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="42">
+        <f>VLOOKUP(B16,DADOS!$B$3:$E$6,MATCH($E$11,DADOS!$B$2:$E$2,0),FALSE)</f>
+        <v>0.05</v>
+      </c>
+      <c r="F16" s="43"/>
     </row>
     <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="39">
-        <f>INDEX(DADOS!$C$3:$E$6,MATCH(B17,DADOS!$B$3:$B$6,0),MATCH($E$11,DADOS!$C$2:$E$2,0))</f>
-        <v>0.2</v>
-      </c>
-      <c r="F17" s="40"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="42">
+        <f>VLOOKUP(B17,DADOS!$B$3:$E$6,MATCH($E$11,DADOS!$B$2:$E$2,0),FALSE)</f>
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="43"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="41">
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="44">
         <f>SUM(E14:E17)</f>
         <v>1</v>
       </c>
-      <c r="F18" s="42"/>
+      <c r="F18" s="45"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C19" s="3"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="B7:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{E0102A38-0475-4B80-AF4E-1F2610E84CEB}">

</xml_diff>